<commit_message>
Additional Unique NPC アビリティの調整
</commit_message>
<xml_diff>
--- a/AdditionalUniqueNPC/package/LangMod/JP/SourceSheet.xlsx
+++ b/AdditionalUniqueNPC/package/LangMod/JP/SourceSheet.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="609" uniqueCount="259">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="606" uniqueCount="256">
   <si>
     <t>id</t>
   </si>
@@ -779,9 +779,6 @@
     <t>Buff</t>
   </si>
   <si>
-    <t>3</t>
-  </si>
-  <si>
     <t>counter,1,evasionPerfect,50</t>
   </si>
   <si>
@@ -791,22 +788,16 @@
     <t>buff</t>
   </si>
   <si>
-    <t>martial</t>
+    <t>AI_Meditate</t>
   </si>
   <si>
     <t>#1は精神を集中させ始めた。</t>
   </si>
   <si>
-    <t>#1 take(s) a counter stance.</t>
-  </si>
-  <si>
     <t>#1は精神の集中を解いた。</t>
   </si>
   <si>
-    <t>#1 leave(s) the counter stance.</t>
-  </si>
-  <si>
-    <t>近接攻撃を高確率で回避し、反撃を行う構え。</t>
+    <t>近接攻撃に対する回避と反撃の能力を向上させる加護。</t>
   </si>
 </sst>
 </file>
@@ -8092,46 +8083,37 @@
         <v>248</v>
       </c>
       <c r="H4" t="s">
+        <v>175</v>
+      </c>
+      <c r="O4" t="s">
         <v>249</v>
       </c>
-      <c r="I4" t="s">
-        <v>249</v>
-      </c>
-      <c r="O4" t="s">
+      <c r="R4" t="s">
         <v>250</v>
       </c>
-      <c r="R4" t="s">
+      <c r="S4" t="s">
         <v>251</v>
       </c>
-      <c r="S4" t="s">
+      <c r="T4" t="s">
         <v>252</v>
       </c>
-      <c r="T4" t="s">
-        <v>253</v>
-      </c>
       <c r="U4" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="V4" t="s">
         <v>215</v>
       </c>
       <c r="X4" t="s">
+        <v>253</v>
+      </c>
+      <c r="Z4" t="s">
         <v>254</v>
-      </c>
-      <c r="Y4" t="s">
-        <v>255</v>
-      </c>
-      <c r="Z4" t="s">
-        <v>256</v>
-      </c>
-      <c r="AA4" t="s">
-        <v>257</v>
       </c>
       <c r="AE4" t="s">
         <v>63</v>
       </c>
       <c r="AF4" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
     </row>
   </sheetData>

</xml_diff>